<commit_message>
[28/10/2026][TrongHieu] Implement UC-01 to UC-07 reusable UI components and widget tests
</commit_message>
<xml_diff>
--- a/EduPlan_Project_Tasks_UC.xlsx
+++ b/EduPlan_Project_Tasks_UC.xlsx
@@ -629,10 +629,10 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>28/10/2026</v>
       </c>
       <c r="F10" t="str">
-        <v>Chưa bắt đầu</v>
+        <v>Đã commit</v>
       </c>
       <c r="G10" t="str">
         <v>Cao 48-52dp, touch target &gt;= 48dp, các state: Default, Pressed, Disabled, Spinner</v>
@@ -652,10 +652,10 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>28/10/2026</v>
       </c>
       <c r="F11" t="str">
-        <v>Chưa bắt đầu</v>
+        <v>Đã commit</v>
       </c>
       <c r="G11" t="str">
         <v>Hiển thị độ khó ⭐, giờ tự học, viền 1px solid, biến thể Conflict viền đỏ 1.5px</v>
@@ -675,10 +675,10 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>28/10/2026</v>
       </c>
       <c r="F12" t="str">
-        <v>Chưa bắt đầu</v>
+        <v>Đã commit</v>
       </c>
       <c r="G12" t="str">
         <v>Ô Search cao 48dp bo góc 8dp, các chip: Tất cả, Chuyên ngành SE, Cơ sở</v>
@@ -698,10 +698,10 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>28/10/2026</v>
       </c>
       <c r="F13" t="str">
-        <v>Chưa bắt đầu</v>
+        <v>Đã commit</v>
       </c>
       <c r="G13" t="str">
         <v>Success (xanh lá #DCFCE7), Warning (vàng nâu #FEF3C7), Danger (đỏ #FEE2E2)</v>
@@ -721,10 +721,10 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>28/10/2026</v>
       </c>
       <c r="F14" t="str">
-        <v>Chưa bắt đầu</v>
+        <v>Đã commit</v>
       </c>
       <c r="G14" t="str">
         <v>Nền đỏ nhạt #FEE2E2, viền đỏ #DC2626, icon ⚠️, chữ đỏ đậm #B91C1C</v>
@@ -744,10 +744,10 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>28/10/2026</v>
       </c>
       <c r="F15" t="str">
-        <v>Chưa bắt đầu</v>
+        <v>Đã commit</v>
       </c>
       <c r="G15" t="str">
         <v>Shimmer xám #EAE1D0; Empty state icon kính lúp + nút "Xóa bộ lọc"</v>
@@ -767,10 +767,10 @@
         <v/>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>28/10/2026</v>
       </c>
       <c r="F16" t="str">
-        <v>Chưa bắt đầu</v>
+        <v>Đã commit</v>
       </c>
       <c r="G16" t="str">
         <v>NavigationBar 64dp 4 tab (Mobile) tự chuyển sang NavigationRail khi width &gt;= 600dp</v>

</xml_diff>

<commit_message>
[28/10/2026][TrongHieu] Implement UC-08 SCR-01 Login screen and loading state
</commit_message>
<xml_diff>
--- a/EduPlan_Project_Tasks_UC.xlsx
+++ b/EduPlan_Project_Tasks_UC.xlsx
@@ -813,10 +813,10 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>28/10/2026</v>
       </c>
       <c r="F18" t="str">
-        <v>Chưa bắt đầu</v>
+        <v>Đã commit</v>
       </c>
       <c r="G18" t="str">
         <v>Logo sổ tay 64dp, slogan, nút đăng nhập Google, spinner "Đang xác thực Google..."</v>

</xml_diff>

<commit_message>
[28/10/2026][TrongHieu] Update project docs, models and services for multi-persona and course progression
</commit_message>
<xml_diff>
--- a/EduPlan_Project_Tasks_UC.xlsx
+++ b/EduPlan_Project_Tasks_UC.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G56"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -827,7 +827,7 @@
         <v>UC-09</v>
       </c>
       <c r="B19" t="str">
-        <v>Xử lý xác thực Google Sign-In &amp; Auth-state Routing (Signed in -&gt; Home)</v>
+        <v>Xử lý Google Sign-In &amp; Đa Persona (3 TK mẫu Long/Linh/Tuấn; TK mới báo rỗng)</v>
       </c>
       <c r="C19" t="str">
         <v>Medium (N=3)</v>
@@ -842,7 +842,7 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G19" t="str">
-        <v>Bắt sự kiện hủy đăng nhập từ người dùng, dọn dẹp session khi sign-out</v>
+        <v>Long (90TC, 34h conflict), Linh (125TC, kỳ tốt nghiệp), Tuấn (35TC, 38h); TK mới báo hồ sơ trống</v>
       </c>
     </row>
     <row r="20">
@@ -942,7 +942,7 @@
         <v>UC-13</v>
       </c>
       <c r="B24" t="str">
-        <v>SCR-03 Màn hình Môn Đã Học (Completed Courses) &amp; Mở khóa tiên quyết</v>
+        <v>SCR-03 Màn hình Môn Đã Học (Completed Courses) &amp; Thẻ tiến độ 90/145 TC</v>
       </c>
       <c r="C24" t="str">
         <v>Medium (N=3)</v>
@@ -962,13 +962,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>UC-14</v>
+        <v>UC-13B</v>
       </c>
       <c r="B25" t="str">
-        <v>SCR-04 Course Catalog: Danh mục môn mở, tìm kiếm &amp; độ khó tự học</v>
+        <v>SCR-03 Modal Thêm môn đã học theo kỳ: Thẩm định kỳ 2 phải có kỳ 1 &amp; Tiên quyết</v>
       </c>
       <c r="C25" t="str">
-        <v>Medium (N=3)</v>
+        <v>Hard (N=5)</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -980,18 +980,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G25" t="str">
-        <v>Thẻ môn học, số TC, độ khó ⭐, tự học h/tuần, nút Tonal Button "Chiến lược &gt;"</v>
+        <v>Nút riêng cho SV tự add môn từng kỳ, validate kỳ 2 phải có kỳ 1 và môn tiên quyết phải hoàn thành trước</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>UC-15</v>
+        <v>UC-14</v>
       </c>
       <c r="B26" t="str">
-        <v>SCR-04 Xử lý Shimmer Skeleton khi tải &amp; Empty State khi tìm kiếm rỗng</v>
+        <v>SCR-04 Course Catalog: Danh mục môn mở, tìm kiếm &amp; độ khó tự học</v>
       </c>
       <c r="C26" t="str">
-        <v>Simple (N=2)</v>
+        <v>Medium (N=3)</v>
       </c>
       <c r="D26" t="str">
         <v/>
@@ -1003,15 +1003,15 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G26" t="str">
-        <v>Khi tìm từ khóa không có môn (VD: XYZ99) hiện kính lúp buồn + nút Xóa bộ lọc</v>
+        <v>Thẻ môn học, số TC, độ khó ⭐, tự học h/tuần, nút Tonal Button "Chiến lược &gt;"</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>UC-16</v>
+        <v>UC-15</v>
       </c>
       <c r="B27" t="str">
-        <v>SCR-05 Course Strategy: Header môn PRM393 &amp; 3 badge thông số</v>
+        <v>SCR-04 Xử lý Shimmer Skeleton khi tải &amp; Empty State khi tìm kiếm rỗng</v>
       </c>
       <c r="C27" t="str">
         <v>Simple (N=2)</v>
@@ -1026,15 +1026,15 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G27" t="str">
-        <v>3 badge: 3 Tín chỉ, Độ khó 4/5 ⭐, Tiên quyết PRO192 ✅. Ẩn hoàn toàn Bottom Bar</v>
+        <v>Khi tìm từ khóa không có môn (VD: XYZ99) hiện kính lúp buồn + nút Xóa bộ lọc</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>UC-17</v>
+        <v>UC-16</v>
       </c>
       <c r="B28" t="str">
-        <v>SCR-05 Cấu trúc điểm 40/30/30 &amp; Thẻ Study Tips khóa trên</v>
+        <v>SCR-05 Course Strategy: Header môn PRM393 &amp; 3 badge thông số</v>
       </c>
       <c r="C28" t="str">
         <v>Simple (N=2)</v>
@@ -1049,18 +1049,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G28" t="str">
-        <v>3 hộp thông số: Đồ án 40%, Lab 30%, FE 30%; Thẻ vàng nhạt tips làm Riverpod/MVVM</v>
+        <v>3 badge: 3 Tín chỉ, Độ khó 4/5 ⭐, Tiên quyết PRO192 ✅. Ẩn hoàn toàn Bottom Bar</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>UC-18</v>
+        <v>UC-17</v>
       </c>
       <c r="B29" t="str">
-        <v>SCR-05 Radio Card chọn Mục tiêu điểm (Điểm A: 8h, B: 5h, Qua môn: 3.5h)</v>
+        <v>SCR-05 Cấu trúc điểm 40/30/30 &amp; Thẻ Study Tips khóa trên</v>
       </c>
       <c r="C29" t="str">
-        <v>Medium (N=3)</v>
+        <v>Simple (N=2)</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -1072,18 +1072,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G29" t="str">
-        <v>3 Radio card tương tác mượt mà, tự động cập nhật số giờ tự học dự kiến</v>
+        <v>3 hộp thông số: Đồ án 40%, Lab 30%, FE 30%; Thẻ vàng nhạt tips làm Riverpod/MVVM</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>UC-19</v>
+        <v>UC-18</v>
       </c>
       <c r="B30" t="str">
-        <v>SCR-05 Docked Action Footer: Nút yêu thích + Nút "Thêm vào Kế hoạch"</v>
+        <v>SCR-05 Radio Card chọn Mục tiêu điểm (Điểm A: 8h, B: 5h, Qua môn: 3.5h)</v>
       </c>
       <c r="C30" t="str">
-        <v>Simple (N=2)</v>
+        <v>Medium (N=3)</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -1095,18 +1095,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G30" t="str">
-        <v>Cố định chân trang, padding-bottom 110dp chống đè nội dung, điều hướng sang SCR-06A</v>
+        <v>3 Radio card tương tác mượt mà, tự động cập nhật số giờ tự học dự kiến</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>NHÓM 4: PHÂN TÍCH QUÁ TẢI &amp; KHẮC PHỤC XUNG ĐỘT (SCR-06A &amp; 06B)</v>
+        <v>UC-19</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v>SCR-05 Docked Action Footer: Nút yêu thích + Nút "Thêm vào Kế hoạch"</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>Simple (N=2)</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -1115,21 +1115,21 @@
         <v/>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>Chưa bắt đầu</v>
       </c>
       <c r="G31" t="str">
-        <v/>
+        <v>Cố định chân trang, padding-bottom 110dp chống đè nội dung, điều hướng sang SCR-06A</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>UC-20</v>
+        <v>NHÓM 4: PHÂN TÍCH QUÁ TẢI &amp; KHẮC PHỤC XUNG ĐỘT (SCR-06A &amp; 06B)</v>
       </c>
       <c r="B32" t="str">
-        <v>SCR-06A Workload Analyzer: Banner cảnh báo đỏ quá tải &amp; vi phạm</v>
+        <v/>
       </c>
       <c r="C32" t="str">
-        <v>Simple (N=2)</v>
+        <v/>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -1138,21 +1138,21 @@
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Chưa bắt đầu</v>
+        <v/>
       </c>
       <c r="G32" t="str">
-        <v>Nền đỏ #FEE2E2, viền #DC2626, icon ⚠️ "Cảnh báo: Vi phạm tiên quyết &amp; Quá tải!"</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>UC-21</v>
+        <v>UC-20</v>
       </c>
       <c r="B33" t="str">
-        <v>SCR-06A Thẻ Workload Meter: 34h/tuần vượt ngưỡng an toàn (25h Remote Config)</v>
+        <v>SCR-06A Workload Analyzer: Banner cảnh báo đỏ quá tải &amp; vi phạm</v>
       </c>
       <c r="C33" t="str">
-        <v>Medium (N=3)</v>
+        <v>Simple (N=2)</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -1164,15 +1164,15 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G33" t="str">
-        <v>Thanh progress bar có đoạn màu đỏ báo quá tải, lấy max_safe_workload_hours động</v>
+        <v>Nền đỏ #FEE2E2, viền #DC2626, icon ⚠️ "Cảnh báo: Vi phạm tiên quyết &amp; Quá tải!"</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>UC-22</v>
+        <v>UC-21</v>
       </c>
       <c r="B34" t="str">
-        <v>SCR-06A Danh sách 4 thẻ môn: 3 môn hợp lệ và 1 môn vi phạm đỏ IAE201</v>
+        <v>SCR-06A Thẻ Workload Meter: 34h/tuần vượt ngưỡng an toàn (25h Remote Config)</v>
       </c>
       <c r="C34" t="str">
         <v>Medium (N=3)</v>
@@ -1187,18 +1187,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G34" t="str">
-        <v>PRM393 (8h), SWE302 (7h), AIE411 (7h); IAE201 (+12h, LỖI chưa học tiên quyết NWC203)</v>
+        <v>Thanh progress bar có đoạn màu đỏ báo quá tải, lấy max_safe_workload_hours động</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>UC-23</v>
+        <v>UC-22</v>
       </c>
       <c r="B35" t="str">
-        <v>SCR-06B Selected Courses (State lỗi): Nút Lưu BỊ KHÓA &amp; Nút [⇄ Đổi môn]</v>
+        <v>SCR-06A Danh sách 4 thẻ môn: 3 môn hợp lệ và 1 môn vi phạm đỏ IAE201</v>
       </c>
       <c r="C35" t="str">
-        <v>Hard (N=5)</v>
+        <v>Medium (N=3)</v>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -1210,15 +1210,15 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G35" t="str">
-        <v>Nút chân trang màu xám "🔒 Giải quyết 1 xung đột để lưu"; nút Đổi môn mở SCR-05</v>
+        <v>PRM393 (8h), SWE302 (7h), AIE411 (7h); IAE201 (+12h, LỖI chưa học tiên quyết NWC203)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>UC-24</v>
+        <v>UC-23</v>
       </c>
       <c r="B36" t="str">
-        <v>SCR-06B_Resolved Khắc phục xung đột: Đổi sang PRM323, tải 26h Cân bằng</v>
+        <v>SCR-06B Selected Courses (State lỗi): Nút Lưu BỊ KHÓA &amp; Nút [⇄ Đổi môn]</v>
       </c>
       <c r="C36" t="str">
         <v>Hard (N=5)</v>
@@ -1233,18 +1233,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G36" t="str">
-        <v>Môn thứ 4 đổi thành PRM323 (4h), tổng 26h; NÚT LƯU MỞ KHÓA MÀU XANH ACTIVE</v>
+        <v>Nút chân trang màu xám "🔒 Giải quyết 1 xung đột để lưu"; nút Đổi môn mở SCR-05</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>UC-25</v>
+        <v>UC-24</v>
       </c>
       <c r="B37" t="str">
-        <v>Lưu Kế hoạch học tập vào Firestore &amp; Chuyển hướng sang SCR-07</v>
+        <v>SCR-06B_Resolved Khắc phục xung đột: Đổi sang PRM323, tải 26h Cân bằng</v>
       </c>
       <c r="C37" t="str">
-        <v>Medium (N=3)</v>
+        <v>Hard (N=5)</v>
       </c>
       <c r="D37" t="str">
         <v/>
@@ -1256,18 +1256,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G37" t="str">
-        <v>Ghi dữ liệu kế hoạch hợp lệ vào study_plans trên Cloud Firestore, pushNamed sang SCR-07</v>
+        <v>Môn thứ 4 đổi thành PRM323 (4h), tổng 26h; NÚT LƯU MỞ KHÓA MÀU XANH ACTIVE</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>NHÓM 5: TỔNG KẾT KẾ HOẠCH &amp; XUẤT BLUEPRINT PDF (SCR-07)</v>
+        <v>UC-25</v>
       </c>
       <c r="B38" t="str">
-        <v/>
+        <v>Lưu Kế hoạch học tập vào Firestore &amp; Chuyển hướng sang SCR-07</v>
       </c>
       <c r="C38" t="str">
-        <v/>
+        <v>Medium (N=3)</v>
       </c>
       <c r="D38" t="str">
         <v/>
@@ -1276,21 +1276,21 @@
         <v/>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>Chưa bắt đầu</v>
       </c>
       <c r="G38" t="str">
-        <v/>
+        <v>Ghi dữ liệu kế hoạch hợp lệ vào study_plans trên Cloud Firestore, pushNamed sang SCR-07</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>UC-26</v>
+        <v>NHÓM 5: TỔNG KẾT KẾ HOẠCH &amp; XUẤT BLUEPRINT PDF (SCR-07)</v>
       </c>
       <c r="B39" t="str">
-        <v>SCR-07 Semester Summary: Thẻ Hero KPI (5 Môn, 15 TC, GPA 3.65, 26h tự học)</v>
+        <v/>
       </c>
       <c r="C39" t="str">
-        <v>Simple (N=2)</v>
+        <v/>
       </c>
       <c r="D39" t="str">
         <v/>
@@ -1299,18 +1299,18 @@
         <v/>
       </c>
       <c r="F39" t="str">
-        <v>Chưa bắt đầu</v>
+        <v/>
       </c>
       <c r="G39" t="str">
-        <v>Khôi phục Bottom Bar; 4 nhãn KPI chia 2 hàng: Lộ trình hợp lệ, Học phí 14.250.000đ</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>UC-27</v>
+        <v>UC-26</v>
       </c>
       <c r="B40" t="str">
-        <v>SCR-07 Danh sách 5 môn học kèm mục tiêu điểm (A / B+) và tích xanh ✅</v>
+        <v>SCR-07 Semester Summary: Thẻ Hero KPI (5 Môn, 15 TC, GPA 3.65, 26h tự học)</v>
       </c>
       <c r="C40" t="str">
         <v>Simple (N=2)</v>
@@ -1325,15 +1325,15 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G40" t="str">
-        <v>Hiển thị PRM393, SWE302, AIE411, PRM323, OSG209 thẻ nhỏ gọn, căn gióng đẹp mắt</v>
+        <v>Khôi phục Bottom Bar; 4 nhãn KPI chia 2 hàng: Lộ trình hợp lệ, Học phí 14.250.000đ</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>UC-28</v>
+        <v>UC-26B</v>
       </c>
       <c r="B41" t="str">
-        <v>SCR-07 Tạo file tài liệu PDF Blueprint A4 Kế hoạch học tập</v>
+        <v>SCR-07 Nút "Đã hoàn thành kỳ học": Tự động lưu các môn vào Môn Đã Học &amp; Tích lũy TC</v>
       </c>
       <c r="C41" t="str">
         <v>Medium (N=4)</v>
@@ -1348,18 +1348,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G41" t="str">
-        <v>Dựng bằng pdf &amp; printing package: Header, bảng KPI, bảng điểm &amp; giờ tự học từng môn</v>
+        <v>Tự động chuyển các môn trong kỳ thành Môn đã hoàn thành, cộng dồn accumulatedCredits và update status</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>UC-29</v>
+        <v>UC-27</v>
       </c>
       <c r="B42" t="str">
-        <v>SCR-07 Upload file PDF lên Firebase Storage reports/{uid}/... &amp; hiển thị progress</v>
+        <v>SCR-07 Danh sách 5 môn học kèm mục tiêu điểm (A / B+) và tích xanh ✅</v>
       </c>
       <c r="C42" t="str">
-        <v>Hard (N=5)</v>
+        <v>Simple (N=2)</v>
       </c>
       <c r="D42" t="str">
         <v/>
@@ -1371,18 +1371,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G42" t="str">
-        <v>Thanh tiến trình % tải lên, lấy download URL thật trên Cloud Storage (bucket Blaze)</v>
+        <v>Hiển thị PRM393, SWE302, AIE411, PRM323, OSG209 thẻ nhỏ gọn, căn gióng đẹp mắt</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>UC-30</v>
+        <v>UC-28</v>
       </c>
       <c r="B43" t="str">
-        <v>SCR-07 Kích hoạt hộp thoại xem trước in ấn PDF &amp; Đồng bộ lịch Google Calendar</v>
+        <v>SCR-07 Tạo file tài liệu PDF Blueprint A4 Kế hoạch học tập</v>
       </c>
       <c r="C43" t="str">
-        <v>Simple (N=2)</v>
+        <v>Medium (N=4)</v>
       </c>
       <c r="D43" t="str">
         <v/>
@@ -1394,18 +1394,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G43" t="str">
-        <v>Nút "📄 Xuất PDF Kế Hoạch &amp; Chiến Lược (A4)", nút Đồng bộ lịch và nút Chia sẻ</v>
+        <v>Dựng bằng pdf &amp; printing package: Header, bảng KPI, bảng điểm &amp; giờ tự học từng môn</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>NHÓM 6: HỒ SƠ CÁ NHÂN &amp; FIREBASE DEMO (SCR-08)</v>
+        <v>UC-29</v>
       </c>
       <c r="B44" t="str">
-        <v/>
+        <v>SCR-07 Upload file PDF lên Firebase Storage reports/{uid}/... &amp; hiển thị progress</v>
       </c>
       <c r="C44" t="str">
-        <v/>
+        <v>Hard (N=5)</v>
       </c>
       <c r="D44" t="str">
         <v/>
@@ -1414,18 +1414,18 @@
         <v/>
       </c>
       <c r="F44" t="str">
-        <v/>
+        <v>Chưa bắt đầu</v>
       </c>
       <c r="G44" t="str">
-        <v/>
+        <v>Thanh tiến trình % tải lên, lấy download URL thật trên Cloud Storage (bucket Blaze)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>UC-31</v>
+        <v>UC-30</v>
       </c>
       <c r="B45" t="str">
-        <v>SCR-08 Profile: Thẻ sinh viên Trần Hoàng Long, MSSV SE180504, GPA 3.42</v>
+        <v>SCR-07 Kích hoạt hộp thoại xem trước in ấn PDF &amp; Đồng bộ lịch Google Calendar</v>
       </c>
       <c r="C45" t="str">
         <v>Simple (N=2)</v>
@@ -1440,18 +1440,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G45" t="str">
-        <v>Avatar tròn, pill Đã tích lũy: 90 / 145 TC và pill ⭐ GPA: 3.42 (Giỏi)</v>
+        <v>Nút "📄 Xuất PDF Kế Hoạch &amp; Chiến Lược (A4)", nút Đồng bộ lịch và nút Chia sẻ</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>UC-32</v>
+        <v>NHÓM 6: HỒ SƠ CÁ NHÂN &amp; FIREBASE DEMO (SCR-08)</v>
       </c>
       <c r="B46" t="str">
-        <v>SCR-08 Thẻ học kỳ Fall 2024: Nút "Chi tiết &gt;" mở lại màn hình SCR-07</v>
+        <v/>
       </c>
       <c r="C46" t="str">
-        <v>Simple (N=1)</v>
+        <v/>
       </c>
       <c r="D46" t="str">
         <v/>
@@ -1460,21 +1460,21 @@
         <v/>
       </c>
       <c r="F46" t="str">
-        <v>Chưa bắt đầu</v>
+        <v/>
       </c>
       <c r="G46" t="str">
-        <v>Touch target 48dp, chuyển hướng mượt mà sang bản tổng kết kế hoạch đã lưu</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>UC-33</v>
+        <v>UC-31</v>
       </c>
       <c r="B47" t="str">
-        <v>SCR-08 Nhóm cài đặt 3 Switch: Nhắc hạn Lab, Cảnh báo quá tải, Sync Calendar</v>
+        <v>SCR-08 Profile: Thẻ sinh viên &amp; Modal Chỉnh sửa hồ sơ (Tên, Ảnh, MSSV, GPA mục tiêu)</v>
       </c>
       <c r="C47" t="str">
-        <v>Simple (N=2)</v>
+        <v>Medium (N=3)</v>
       </c>
       <c r="D47" t="str">
         <v/>
@@ -1486,18 +1486,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G47" t="str">
-        <v>Chiều cao mỗi tile &gt;= 56dp, đồng bộ trạng thái toggle tức thời lên Cloud Firestore</v>
+        <v>Avatar tròn, nút Chỉnh sửa hồ sơ, modal cập nhật Họ tên, MSSV, ảnh đại diện, GPA mục tiêu lên Firestore</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>UC-34</v>
+        <v>UC-32</v>
       </c>
       <c r="B48" t="str">
-        <v>SCR-08 Firebase Demo Showcase: Crashlytics test, Remote Config &amp; FCM inbox</v>
+        <v>SCR-08 Thẻ học kỳ Fall 2024: Nút "Chi tiết &gt;" mở lại màn hình SCR-07</v>
       </c>
       <c r="C48" t="str">
-        <v>Medium (N=4)</v>
+        <v>Simple (N=1)</v>
       </c>
       <c r="D48" t="str">
         <v/>
@@ -1509,15 +1509,15 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G48" t="str">
-        <v>Nút test Crashlytics (non-fatal error &amp; crash), hiển thị giá trị Remote Config động</v>
+        <v>Touch target 48dp, chuyển hướng mượt mà sang bản tổng kết kế hoạch đã lưu</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>UC-35</v>
+        <v>UC-33</v>
       </c>
       <c r="B49" t="str">
-        <v>Overlay_Logout Modal: Hộp thoại xác nhận đăng xuất tài khoản</v>
+        <v>SCR-08 Nhóm cài đặt 3 Switch: Nhắc hạn Lab, Cảnh báo quá tải, Sync Calendar</v>
       </c>
       <c r="C49" t="str">
         <v>Simple (N=2)</v>
@@ -1532,18 +1532,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G49" t="str">
-        <v>Dialog 320dp bo góc 16dp, 2 nút Hủy và Đăng xuất (50/50), xóa session về SCR-01</v>
+        <v>Chiều cao mỗi tile &gt;= 56dp, đồng bộ trạng thái toggle tức thời lên Cloud Firestore</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>NHÓM 7: ĐO LƯỜNG SỰ KIỆN &amp; KIỂM THỬ E2E (Analytics &amp; Testing)</v>
+        <v>UC-34</v>
       </c>
       <c r="B50" t="str">
-        <v/>
+        <v>SCR-08 Firebase Demo Showcase: Crashlytics test, Remote Config &amp; FCM inbox</v>
       </c>
       <c r="C50" t="str">
-        <v/>
+        <v>Medium (N=4)</v>
       </c>
       <c r="D50" t="str">
         <v/>
@@ -1552,21 +1552,21 @@
         <v/>
       </c>
       <c r="F50" t="str">
-        <v/>
+        <v>Chưa bắt đầu</v>
       </c>
       <c r="G50" t="str">
-        <v/>
+        <v>Nút test Crashlytics (non-fatal error &amp; crash), hiển thị giá trị Remote Config động</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>UC-36</v>
+        <v>UC-35</v>
       </c>
       <c r="B51" t="str">
-        <v>Gắn mã ghi nhận 8 sự kiện Firebase Analytics (DebugView verification)</v>
+        <v>Overlay_Logout Modal: Hộp thoại xác nhận đăng xuất tài khoản</v>
       </c>
       <c r="C51" t="str">
-        <v>Medium (N=3)</v>
+        <v>Simple (N=2)</v>
       </c>
       <c r="D51" t="str">
         <v/>
@@ -1578,18 +1578,18 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G51" t="str">
-        <v>Đầy đủ parameters không PII: login, search, view_detail, conflict, resolve, export...</v>
+        <v>Dialog 320dp bo góc 16dp, 2 nút Hủy và Đăng xuất (50/50), xóa session về SCR-01</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>UC-37</v>
+        <v>NHÓM 7: ĐO LƯỜNG SỰ KIỆN &amp; KIỂM THỬ E2E (Analytics &amp; Testing)</v>
       </c>
       <c r="B52" t="str">
-        <v>Gắn Semantics Labels trợ năng cho toàn bộ nút bấm, card, ô nhập liệu</v>
+        <v/>
       </c>
       <c r="C52" t="str">
-        <v>Simple (N=2)</v>
+        <v/>
       </c>
       <c r="D52" t="str">
         <v/>
@@ -1598,21 +1598,21 @@
         <v/>
       </c>
       <c r="F52" t="str">
-        <v>Chưa bắt đầu</v>
+        <v/>
       </c>
       <c r="G52" t="str">
-        <v>Phục vụ khả năng tiếp cận WCAG và giúp AI Agent ARTEMIS đọc cây widget</v>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>UC-38</v>
+        <v>UC-36</v>
       </c>
       <c r="B53" t="str">
-        <v>Xây dựng kịch bản kiểm thử E2E tự động với Google ARTEMIS / Pytest</v>
+        <v>Gắn mã ghi nhận 8 sự kiện Firebase Analytics (DebugView verification)</v>
       </c>
       <c r="C53" t="str">
-        <v>Hard (N=6)</v>
+        <v>Medium (N=3)</v>
       </c>
       <c r="D53" t="str">
         <v/>
@@ -1624,35 +1624,81 @@
         <v>Chưa bắt đầu</v>
       </c>
       <c r="G53" t="str">
-        <v>&gt;= 10 test cases trong e2e_test/, bao gồm luồng chính, native dialog và error-path</v>
+        <v>Đầy đủ parameters không PII: login, search, view_detail, conflict, resolve, export...</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
+        <v>UC-37</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Gắn Semantics Labels trợ năng cho toàn bộ nút bấm, card, ô nhập liệu</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Simple (N=2)</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v>Chưa bắt đầu</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Phục vụ khả năng tiếp cận WCAG và giúp AI Agent ARTEMIS đọc cây widget</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>UC-38</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Xây dựng kịch bản kiểm thử E2E tự động với Google ARTEMIS / Pytest</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Hard (N=6)</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v>Chưa bắt đầu</v>
+      </c>
+      <c r="G55" t="str">
+        <v>&gt;= 10 test cases trong e2e_test/, bao gồm luồng chính, native dialog và error-path</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
         <v>UC-39</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B56" t="str">
         <v>Thực hiện AI-Assisted Code Review &amp; lưu bằng chứng docs/code-review.md</v>
       </c>
-      <c r="C54" t="str">
+      <c r="C56" t="str">
         <v>Medium (N=3)</v>
       </c>
-      <c r="D54" t="str">
-        <v/>
-      </c>
-      <c r="E54" t="str">
-        <v/>
-      </c>
-      <c r="F54" t="str">
-        <v>Chưa bắt đầu</v>
-      </c>
-      <c r="G54" t="str">
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v>Chưa bắt đầu</v>
+      </c>
+      <c r="G56" t="str">
         <v>Ghi nhận &gt;= 5 findings, ra quyết định chấp nhận/từ chối và &gt;= 3 commit sửa lỗi</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G56"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>